<commit_message>
TD-D86-002 + TD-D86-006: контроль условий Table 5 (d86_procedure) и GUM-модель D86 (evaluate_gum_d86); book-слой: листы GUM_u(T)+Условия_Table5 в ASTM v3.13; тесты+доки
</commit_message>
<xml_diff>
--- a/new_versions_v4.2/ASTM_D86_ручной_метод_v3.13_контракт_с_генератором.xlsx
+++ b/new_versions_v4.2/ASTM_D86_ручной_метод_v3.13_контракт_с_генератором.xlsx
@@ -14,7 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Аудит_НД" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Техдолг" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракт_v313" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр_НД" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUM_u(T)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Условия_Table5" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр_НД" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Аудит_НД'!$A$1:$G$11</definedName>
@@ -1663,6 +1665,624 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>КОНТРОЛЬ УСЛОВИЙ ИСПЫТАНИЯ ASTM D86-23 TABLE 5 — fraction_lib.d86_procedure (TD-D86-002)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Источник чисел:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>python -m fraction_lib.excel_generator (лист генерируется, не редактировать вручную)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ОГОВОРКА: справочник ниже — типовая сводка Table 5; до ввода в эксплуатацию сверить</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>с лицензионной копией ASTM D86-23 (реестр НД, лист «Реестр_НД»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>= 1. Справочник Table 5 (по группам продукта) ==</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Группа</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Продукты</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Объём пробы, мл</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Конденсация, мл/мин</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>IBP→5%, мин</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Нагрев до IBP, мин</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Лёгкие продукты (бензины)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>99.5–100.5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4.0–5.0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>≤ 10.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>≤ 10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Топки и средние дистилляты (авиакеросин, дизель)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>99.5–100.5</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4.0–5.0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>≤ 10.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>≤ 10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Газойли и тяжёлые дистилляты</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>99.5–100.5</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4.0–5.0</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Тяжёлые продукты (мазуты, битумные фракции)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>99.5–100.5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.001–5.0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>= 2. Вердикт по эталонным данным листа «Ввод» ==</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Группа из «Ввод»:</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>| Объём пробы, мл:</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Вердикт:</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Флаги policy:</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>WARNING:TABLE5:CONDENSE_RATE, WARNING:TABLE5:BATH_PREHEAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Требование</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Факт</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CONDENSE_RATE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Скорость конденсации гр.4: 0.001–5.0 мл/мин</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BATH_PREHEAT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Баня/нагрев прогреты по Table 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Правила: MISSING/INVALID =&gt; FAIL (расчёт не пригоден к отчёту без повторного</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>определения или обоснования метролога); WARNING =&gt; CONDITIONAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Поля CONDENSE_RATE / IBP_TO_5 / TIME_TO_IBP / BATH_PREHEAT заполняются оператором</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>из журнала испытания; при regeneration они подхватятся из листа «Ввод», когда</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>колонки будут добавлены (остаток долга — процедуры TD-D86-003/004).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>РЕЕСТР РЕДАКЦИЙ НД (docs/ND_REGISTRY.json) — TD-2177-008 / TD-D86-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Эта книга верифицирована редакцией:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ASTM D86</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Статус сверки хешей (drift-guard):</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>OK — константы кода соответствуют реестру</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Обозначение</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Редакция</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Действует с</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Заменяет</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>sha256 нормативного ядра</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Верифицировано (доказательства)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Область</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ND-2026-001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ГОСТ 2177-99</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Изм. №1 (введён 01.07.2021, приказ 896-ст) + Поправка 2023</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>5b143c2b4b5090e6c3dc5141fd350c40fc6270a7e1cc1655f1bce146894effe9</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>fraction_lib/tests/test_gost2177.py; fraction_lib/tests/test_uncertainty_td2177007.py; fraction_lib/tests/test_procedure_td2177006.py; docs/TECHDEBT_TD2177_002.md; docs/TECHDEBT_TD2177_004.md; docs/TECHDEBT_TD2177_005.md; docs/TECHDEBT_TD2177_007.md</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>fraction_lib.gost2177, fraction_lib.uncertainty, fraction_lib.procedure; книги ГОСТ_2177_метод_А v3.12/v3.13</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>kPa-форма 0.0009*(101.3-p)*(273+t) эквивалентна нормативной 0.0000009*(101300-Pb)*(273+t) — осознанно не менялась (аудит G2177-N03).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ND-2026-002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ASTM D86</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>D86-23 (+ae1)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2023-06-01</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9d600b919fec365ed73df472b37227bc42f2f66035592abc312d45920028a67d</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>fraction_lib/tests/test_d86.py; fraction_lib/tests/test_excel_contract.py; docs (лист Аудит_НД книги v3.12)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>fraction_lib.d86; книги ASTM_D86_ручной_метод v3.12/v3.13; автоматический метод v3.11 (частично)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Единая формула Lc для P&gt;760 внедрена в v3.12 и fraction_lib (TD-D86-001 часть book закрыта коммитом 1322c85). Сингулярность P≈820 мм рт. ст. — warning-слой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ND-LEGACY-001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ASTM D86</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>D86-20a</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2020-01-01</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>исторические книги v3.11 и раннее</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Заменена на ND-2026-002 (D86-23). Расчёт по этой редакции запрещён resolve_for_calculation().</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Правила: запись неизменяема; новая редакция = новая запись + supersedes;</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>расчёт по WITHDRAWN/SUPERSEDED запрещён (resolve_for_calculation);</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>изменение существенных констант без переоформления реестра блокирует CI (pytest).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -8640,252 +9260,1295 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>РЕЕСТР РЕДАКЦИЙ НД (docs/ND_REGISTRY.json) — TD-2177-008 / TD-D86-007</t>
+          <t>GUM-МОДЕЛЬ НЕОПРЕДЕЛЁННОСТИ T_c(V) — fraction_lib.uncertainty.evaluate_gum_d86 (TD-D86-006)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Эта книга верифицирована редакцией:</t>
+          <t>Модель:</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASTM D86</t>
+          <t>T_c = T_obs + 0.00012*(760-P_mm)*(273+t_bar) + ΔT_loss; отчёт округлён до 0.5 °C</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Статус сверки хешей (drift-guard):</t>
+          <t>Источник чисел:</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OK — константы кода соответствуют реестру</t>
+          <t>python -m fraction_lib.excel_generator (лист генерируется, не редактировать вручную)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Условия прогона:</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P = 755.0 мм рт.ст.;</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>t_bar = 20.0 °C (при отсутствии ввода принят 20 °C);</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>объём пробы = 100.0 мл;</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>флаги политики: (нет)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Обозначение</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Редакция</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Действует с</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Заменяет</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>sha256 нормативного ядра</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Верифицировано (доказательства)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Область</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Примечание</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ND-2026-001</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ГОСТ 2177-99</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Изм. №1 (введён 01.07.2021, приказ 896-ст) + Поправка 2023</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2021-07-01</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>5b143c2b4b5090e6c3dc5141fd350c40fc6270a7e1cc1655f1bce146894effe9</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>fraction_lib/tests/test_gost2177.py; fraction_lib/tests/test_uncertainty_td2177007.py; fraction_lib/tests/test_procedure_td2177006.py; docs/TECHDEBT_TD2177_002.md; docs/TECHDEBT_TD2177_004.md; docs/TECHDEBT_TD2177_005.md; docs/TECHDEBT_TD2177_007.md</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>fraction_lib.gost2177, fraction_lib.uncertainty, fraction_lib.procedure; книги ГОСТ_2177_метод_А v3.12/v3.13</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>kPa-форма 0.0009*(101.3-p)*(273+t) эквивалентна нормативной 0.0000009*(101300-Pb)*(273+t) — осознанно не менялась (аудит G2177-N03).</t>
-        </is>
+      <c r="A6">
+        <f>= 1. Компоненты бюджета (пример: точка 50 %, slope как чувствительность объёма) ==</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ND-2026-002</t>
+          <t>Код</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASTM D86</t>
+          <t>Описание</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>D86-23 (+ae1)</t>
+          <t>Тип</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>Распределение</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2023-06-01</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>Полуширина</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9d600b919fec365ed73df472b37227bc42f2f66035592abc312d45920028a67d</t>
+          <t>Чувствительность c_i</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>fraction_lib/tests/test_d86.py; fraction_lib/tests/test_excel_contract.py; docs (лист Аудит_НД книги v3.12)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>fraction_lib.d86; книги ASTM_D86_ручной_метод v3.12/v3.13; автоматический метод v3.11 (частично)</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Единая формула Lc для P&gt;760 внедрена в v3.12 и fraction_lib (TD-D86-001 часть book закрыта коммитом 1322c85). Сингулярность P≈820 мм рт. ст. — warning-слой.</t>
+          <t>u_i, °C</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ND-LEGACY-001</t>
+          <t>u1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ASTM D86</t>
+          <t>Наблюдение T_obs (цена деления, прямоугольный)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>D86-20a</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2020-01-01</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>исторические книги v3.11 и раннее</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Заменена на ND-2026-002 (D86-23). Расчёт по этой редакции запрещён resolve_for_calculation().</t>
-        </is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.2887</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>u2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Барометрическое давление P (Янг)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>мм рт.ст.</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>-0.03516</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.0101</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Правила: запись неизменяема; новая редакция = новая запись + supersedes;</t>
-        </is>
+          <t>u3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Температура барометра t_bar</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.0002</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>расчёт по WITHDRAWN/SUPERSEDED запрещён (resolve_for_calculation);</t>
-        </is>
+          <t>u4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Мениск / выступающий столбик термометра</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.2887</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>изменение существенных констант без переоформления реестра блокирует CI (pytest).</t>
+          <t>u5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Отсчёт объёма V (через локальный slope)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>мл</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1.20072</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.3466</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>u6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Коррекция потерь/остатка ΔT_loss</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.2887</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>u7</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Округление отчёта до 0.5 °C</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>rectangular</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.1443</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>u_c (комбинированная), °C:</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.6254</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>k использованный:</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>| ν_eff:</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>| t95(ν_eff):</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>U = k·u_c, °C:</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.2507</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>valid_for_reporting:</t>
+        </is>
+      </c>
+      <c r="B19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <f>= 2. Сквозной профиль U по точкам книги ==</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>% отгона</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>T_corr_ref, °C</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>slope, °C/%</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>u_c, °C</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>U, °C</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ν_eff</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>t95</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>valid_for_reporting</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Компоненты u_i (°C)</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Замечания</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>0</v>
+      </c>
+      <c r="B23" t="n">
+        <v>162.01085</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5.753</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.741</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3.481</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=1.661, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="n">
+        <v>190.7781</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4.203</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I24" t="b">
+        <v>1</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=1.213, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B25" t="n">
+        <v>204.03605</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.951</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.534</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.563, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B26" t="n">
+        <v>210.2898</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2.376</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.686, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" t="n">
+        <v>227.8003</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2.501</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.722, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="n">
+        <v>235.3048</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.651</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.412</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I28" t="b">
+        <v>1</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.477, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>30</v>
+      </c>
+      <c r="B29" t="n">
+        <v>244.3102</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.501</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.677</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.433, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>35</v>
+      </c>
+      <c r="B30" t="n">
+        <v>250.3138</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1.251</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.267</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.361, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>40</v>
+      </c>
+      <c r="B31" t="n">
+        <v>256.8177</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1.201</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.251</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.347, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>45</v>
+      </c>
+      <c r="B32" t="n">
+        <v>262.321</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1.226</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.629</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.259</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.354, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>50</v>
+      </c>
+      <c r="B33" t="n">
+        <v>269.07505</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1.201</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.251</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.347, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>55</v>
+      </c>
+      <c r="B34" t="n">
+        <v>274.3282</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.176</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.243</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I34" t="b">
+        <v>1</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.339, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>60</v>
+      </c>
+      <c r="B35" t="n">
+        <v>280.8321</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1.301</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1.284</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.376, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>65</v>
+      </c>
+      <c r="B36" t="n">
+        <v>287.336</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1.326</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.646</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1.292</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I36" t="b">
+        <v>1</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.383, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>70</v>
+      </c>
+      <c r="B37" t="n">
+        <v>294.09005</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1.301</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.284</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I37" t="b">
+        <v>1</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.376, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>75</v>
+      </c>
+      <c r="B38" t="n">
+        <v>300.3438</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1.551</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.6870000000000001</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.373</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I38" t="b">
+        <v>1</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.448, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>80</v>
+      </c>
+      <c r="B39" t="n">
+        <v>309.59935</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1.801</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1.471</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I39" t="b">
+        <v>1</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.52, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>85</v>
+      </c>
+      <c r="B40" t="n">
+        <v>318.3546</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2.051</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.577</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I40" t="b">
+        <v>1</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.592, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>90</v>
+      </c>
+      <c r="B41" t="n">
+        <v>330.11165</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2.727</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.887</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I41" t="b">
+        <v>1</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.787, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>95</v>
+      </c>
+      <c r="B42" t="n">
+        <v>345.62095</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2.527</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.792</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I42" t="b">
+        <v>1</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.729, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>100</v>
+      </c>
+      <c r="B43" t="n">
+        <v>355.3768</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1.951</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.534</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I43" t="b">
+        <v>1</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>u1=0.289, u2=0.01, u3=0.0, u4=0.289, u5=0.563, u6=0.289, u7=0.144</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Как использовать: U из этого листа — расширенная неопределённость скорректированной</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>температуры отгона D86; применять вместе с флагами листа «Контракт_v313» и вердиктом</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>листа «Условия_Table5». valid_for_reporting=FALSE = точка получена вне канона НД.</t>
         </is>
       </c>
     </row>

</xml_diff>